<commit_message>
test ok avec fichier cycle
</commit_message>
<xml_diff>
--- a/data/Rename_columns.xlsx
+++ b/data/Rename_columns.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D521"/>
+  <dimension ref="A1:D525"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="25.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -1446,7 +1446,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>centre analytique</t>
+          <t>centre_cout</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1454,10 +1454,8 @@
           <t>Standard</t>
         </is>
       </c>
-      <c r="D44" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
+      <c r="D44" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="45">
@@ -1512,7 +1510,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>centre analytique</t>
+          <t>centre_cout</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -1520,10 +1518,8 @@
           <t>Standard</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
-        <is>
-          <t>False</t>
-        </is>
+      <c r="D47" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="48">
@@ -7966,12 +7962,12 @@
       </c>
       <c r="B342" t="inlineStr">
         <is>
-          <t>date_operation</t>
+          <t>date_saisie</t>
         </is>
       </c>
       <c r="C342" t="inlineStr">
         <is>
-          <t>Perfect Vision</t>
+          <t>Standard</t>
         </is>
       </c>
       <c r="D342" t="b">
@@ -8726,7 +8722,7 @@
       </c>
       <c r="B380" t="inlineStr">
         <is>
-          <t>devise</t>
+          <t>code_devise</t>
         </is>
       </c>
       <c r="C380" t="inlineStr">
@@ -11555,6 +11551,86 @@
         </is>
       </c>
       <c r="D521" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="522">
+      <c r="A522" t="inlineStr">
+        <is>
+          <t>code_centre_cout</t>
+        </is>
+      </c>
+      <c r="B522" t="inlineStr">
+        <is>
+          <t>centre_cout</t>
+        </is>
+      </c>
+      <c r="C522" t="inlineStr">
+        <is>
+          <t>Perfect Vision</t>
+        </is>
+      </c>
+      <c r="D522" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="523">
+      <c r="A523" t="inlineStr">
+        <is>
+          <t>Numero de la piece d'identite</t>
+        </is>
+      </c>
+      <c r="B523" t="inlineStr">
+        <is>
+          <t>Num?ro de la pi?ce d?identit?</t>
+        </is>
+      </c>
+      <c r="C523" t="inlineStr">
+        <is>
+          <t>Perfect Vision</t>
+        </is>
+      </c>
+      <c r="D523" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="524">
+      <c r="A524" t="inlineStr">
+        <is>
+          <t>numero_piece_identite</t>
+        </is>
+      </c>
+      <c r="B524" t="inlineStr">
+        <is>
+          <t>Num?ro de la pi?ce d?identit?</t>
+        </is>
+      </c>
+      <c r="C524" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="D524" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="525">
+      <c r="A525" t="inlineStr">
+        <is>
+          <t>Mode Desabonne</t>
+        </is>
+      </c>
+      <c r="B525" t="inlineStr">
+        <is>
+          <t>Mode D?sabonn?</t>
+        </is>
+      </c>
+      <c r="C525" t="inlineStr">
+        <is>
+          <t>Standard</t>
+        </is>
+      </c>
+      <c r="D525" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
SQL server et streamlit un
</commit_message>
<xml_diff>
--- a/data/Rename_columns.xlsx
+++ b/data/Rename_columns.xlsx
@@ -491,7 +491,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D525"/>
+  <dimension ref="A1:D577"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15"/>
   <cols>
     <col width="25.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -9322,12 +9322,12 @@
       </c>
       <c r="B410" t="inlineStr">
         <is>
-          <t>ID_POINT_SERVICE</t>
+          <t>point_service</t>
         </is>
       </c>
       <c r="C410" t="inlineStr">
         <is>
-          <t>Perfect Vision - colonne conservee</t>
+          <t>Perfect Vision</t>
         </is>
       </c>
       <c r="D410" t="b">
@@ -9382,12 +9382,12 @@
       </c>
       <c r="B413" t="inlineStr">
         <is>
-          <t>ID_TYPE_OPERATION</t>
+          <t>type_operation</t>
         </is>
       </c>
       <c r="C413" t="inlineStr">
         <is>
-          <t>Perfect Vision - colonne conservee</t>
+          <t>Perfect Vision</t>
         </is>
       </c>
       <c r="D413" t="b">
@@ -11632,6 +11632,1054 @@
       </c>
       <c r="D525" t="b">
         <v>0</v>
+      </c>
+    </row>
+    <row r="526">
+      <c r="A526" t="inlineStr">
+        <is>
+          <t>analyse_source</t>
+        </is>
+      </c>
+      <c r="B526" t="inlineStr">
+        <is>
+          <t>analyse</t>
+        </is>
+      </c>
+      <c r="C526" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D526" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="527">
+      <c r="A527" t="inlineStr">
+        <is>
+          <t>type_ligne</t>
+        </is>
+      </c>
+      <c r="B527" t="inlineStr">
+        <is>
+          <t>type_element</t>
+        </is>
+      </c>
+      <c r="C527" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D527" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="528">
+      <c r="A528" t="inlineStr">
+        <is>
+          <t>ligne_excel</t>
+        </is>
+      </c>
+      <c r="B528" t="inlineStr">
+        <is>
+          <t>ligne_reporting</t>
+        </is>
+      </c>
+      <c r="C528" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D528" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="529">
+      <c r="A529" t="inlineStr">
+        <is>
+          <t>source_donnee</t>
+        </is>
+      </c>
+      <c r="B529" t="inlineStr">
+        <is>
+          <t>origine_donnee</t>
+        </is>
+      </c>
+      <c r="C529" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D529" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="530">
+      <c r="A530" t="inlineStr">
+        <is>
+          <t>source_declaration</t>
+        </is>
+      </c>
+      <c r="B530" t="inlineStr">
+        <is>
+          <t>origine_declaration</t>
+        </is>
+      </c>
+      <c r="C530" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D530" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="531">
+      <c r="A531" t="inlineStr">
+        <is>
+          <t>statut_revue_conformite</t>
+        </is>
+      </c>
+      <c r="B531" t="inlineStr">
+        <is>
+          <t>statut_revue</t>
+        </is>
+      </c>
+      <c r="C531" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D531" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="532">
+      <c r="A532" t="inlineStr">
+        <is>
+          <t>etat_alerte</t>
+        </is>
+      </c>
+      <c r="B532" t="inlineStr">
+        <is>
+          <t>etat</t>
+        </is>
+      </c>
+      <c r="C532" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D532" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="533">
+      <c r="A533" t="inlineStr">
+        <is>
+          <t>description_alerte</t>
+        </is>
+      </c>
+      <c r="B533" t="inlineStr">
+        <is>
+          <t>description</t>
+        </is>
+      </c>
+      <c r="C533" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D533" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="534">
+      <c r="A534" t="inlineStr">
+        <is>
+          <t>motif_etat</t>
+        </is>
+      </c>
+      <c r="B534" t="inlineStr">
+        <is>
+          <t>motif</t>
+        </is>
+      </c>
+      <c r="C534" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D534" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="535">
+      <c r="A535" t="inlineStr">
+        <is>
+          <t>reference_operation_perfect</t>
+        </is>
+      </c>
+      <c r="B535" t="inlineStr">
+        <is>
+          <t>numero_operation</t>
+        </is>
+      </c>
+      <c r="C535" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D535" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="536">
+      <c r="A536" t="inlineStr">
+        <is>
+          <t>id_operation_lab</t>
+        </is>
+      </c>
+      <c r="B536" t="inlineStr">
+        <is>
+          <t>numero_operation</t>
+        </is>
+      </c>
+      <c r="C536" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D536" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="537">
+      <c r="A537" t="inlineStr">
+        <is>
+          <t>identifiant_liste</t>
+        </is>
+      </c>
+      <c r="B537" t="inlineStr">
+        <is>
+          <t>reference_liste</t>
+        </is>
+      </c>
+      <c r="C537" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D537" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="538">
+      <c r="A538" t="inlineStr">
+        <is>
+          <t>id_cloture_compte</t>
+        </is>
+      </c>
+      <c r="B538" t="inlineStr">
+        <is>
+          <t>reference_cloture</t>
+        </is>
+      </c>
+      <c r="C538" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D538" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="539">
+      <c r="A539" t="inlineStr">
+        <is>
+          <t>id_arrete_caisse</t>
+        </is>
+      </c>
+      <c r="B539" t="inlineStr">
+        <is>
+          <t>reference_arrete</t>
+        </is>
+      </c>
+      <c r="C539" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D539" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="540">
+      <c r="A540" t="inlineStr">
+        <is>
+          <t>id_cycle_tontine</t>
+        </is>
+      </c>
+      <c r="B540" t="inlineStr">
+        <is>
+          <t>reference_cycle</t>
+        </is>
+      </c>
+      <c r="C540" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D540" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="541">
+      <c r="A541" t="inlineStr">
+        <is>
+          <t>id_depart_adherent</t>
+        </is>
+      </c>
+      <c r="B541" t="inlineStr">
+        <is>
+          <t>reference_depart</t>
+        </is>
+      </c>
+      <c r="C541" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D541" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="542">
+      <c r="A542" t="inlineStr">
+        <is>
+          <t>JOB_EXECUTION_ID</t>
+        </is>
+      </c>
+      <c r="B542" t="inlineStr">
+        <is>
+          <t>reference_execution</t>
+        </is>
+      </c>
+      <c r="C542" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D542" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="543">
+      <c r="A543" t="inlineStr">
+        <is>
+          <t>id_mouvement</t>
+        </is>
+      </c>
+      <c r="B543" t="inlineStr">
+        <is>
+          <t>reference_mouvement</t>
+        </is>
+      </c>
+      <c r="C543" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D543" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="544">
+      <c r="A544" t="inlineStr">
+        <is>
+          <t>analyse</t>
+        </is>
+      </c>
+      <c r="B544" t="inlineStr">
+        <is>
+          <t>analyse</t>
+        </is>
+      </c>
+      <c r="C544" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D544" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="545">
+      <c r="A545" t="inlineStr">
+        <is>
+          <t>type_element</t>
+        </is>
+      </c>
+      <c r="B545" t="inlineStr">
+        <is>
+          <t>type_element</t>
+        </is>
+      </c>
+      <c r="C545" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D545" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="546">
+      <c r="A546" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+      <c r="B546" t="inlineStr">
+        <is>
+          <t>section</t>
+        </is>
+      </c>
+      <c r="C546" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D546" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="547">
+      <c r="A547" t="inlineStr">
+        <is>
+          <t>ligne_reporting</t>
+        </is>
+      </c>
+      <c r="B547" t="inlineStr">
+        <is>
+          <t>ligne_reporting</t>
+        </is>
+      </c>
+      <c r="C547" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D547" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="548">
+      <c r="A548" t="inlineStr">
+        <is>
+          <t>rubrique</t>
+        </is>
+      </c>
+      <c r="B548" t="inlineStr">
+        <is>
+          <t>rubrique</t>
+        </is>
+      </c>
+      <c r="C548" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D548" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="549">
+      <c r="A549" t="inlineStr">
+        <is>
+          <t>date_evenement</t>
+        </is>
+      </c>
+      <c r="B549" t="inlineStr">
+        <is>
+          <t>date_evenement</t>
+        </is>
+      </c>
+      <c r="C549" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D549" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="550">
+      <c r="A550" t="inlineStr">
+        <is>
+          <t>numero_alerte</t>
+        </is>
+      </c>
+      <c r="B550" t="inlineStr">
+        <is>
+          <t>numero_alerte</t>
+        </is>
+      </c>
+      <c r="C550" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D550" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="551">
+      <c r="A551" t="inlineStr">
+        <is>
+          <t>reference_interne</t>
+        </is>
+      </c>
+      <c r="B551" t="inlineStr">
+        <is>
+          <t>reference_interne</t>
+        </is>
+      </c>
+      <c r="C551" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D551" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="552">
+      <c r="A552" t="inlineStr">
+        <is>
+          <t>reference_externe</t>
+        </is>
+      </c>
+      <c r="B552" t="inlineStr">
+        <is>
+          <t>reference_externe</t>
+        </is>
+      </c>
+      <c r="C552" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D552" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="553">
+      <c r="A553" t="inlineStr">
+        <is>
+          <t>numero_operation</t>
+        </is>
+      </c>
+      <c r="B553" t="inlineStr">
+        <is>
+          <t>numero_operation</t>
+        </is>
+      </c>
+      <c r="C553" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D553" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="554">
+      <c r="A554" t="inlineStr">
+        <is>
+          <t>etat</t>
+        </is>
+      </c>
+      <c r="B554" t="inlineStr">
+        <is>
+          <t>etat</t>
+        </is>
+      </c>
+      <c r="C554" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D554" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="555">
+      <c r="A555" t="inlineStr">
+        <is>
+          <t>statut_revue</t>
+        </is>
+      </c>
+      <c r="B555" t="inlineStr">
+        <is>
+          <t>statut_revue</t>
+        </is>
+      </c>
+      <c r="C555" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D555" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="556">
+      <c r="A556" t="inlineStr">
+        <is>
+          <t>statut_couverture</t>
+        </is>
+      </c>
+      <c r="B556" t="inlineStr">
+        <is>
+          <t>statut_couverture</t>
+        </is>
+      </c>
+      <c r="C556" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D556" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="557">
+      <c r="A557" t="inlineStr">
+        <is>
+          <t>origine_declaration</t>
+        </is>
+      </c>
+      <c r="B557" t="inlineStr">
+        <is>
+          <t>origine_declaration</t>
+        </is>
+      </c>
+      <c r="C557" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D557" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="558">
+      <c r="A558" t="inlineStr">
+        <is>
+          <t>volume</t>
+        </is>
+      </c>
+      <c r="B558" t="inlineStr">
+        <is>
+          <t>volume</t>
+        </is>
+      </c>
+      <c r="C558" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D558" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="559">
+      <c r="A559" t="inlineStr">
+        <is>
+          <t>nombre</t>
+        </is>
+      </c>
+      <c r="B559" t="inlineStr">
+        <is>
+          <t>nombre</t>
+        </is>
+      </c>
+      <c r="C559" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D559" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="560">
+      <c r="A560" t="inlineStr">
+        <is>
+          <t>profil_risque</t>
+        </is>
+      </c>
+      <c r="B560" t="inlineStr">
+        <is>
+          <t>profil_risque</t>
+        </is>
+      </c>
+      <c r="C560" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D560" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="561">
+      <c r="A561" t="inlineStr">
+        <is>
+          <t>severite</t>
+        </is>
+      </c>
+      <c r="B561" t="inlineStr">
+        <is>
+          <t>severite</t>
+        </is>
+      </c>
+      <c r="C561" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D561" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="562">
+      <c r="A562" t="inlineStr">
+        <is>
+          <t>action_recommandee</t>
+        </is>
+      </c>
+      <c r="B562" t="inlineStr">
+        <is>
+          <t>action_recommandee</t>
+        </is>
+      </c>
+      <c r="C562" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D562" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="563">
+      <c r="A563" t="inlineStr">
+        <is>
+          <t>origine_donnee</t>
+        </is>
+      </c>
+      <c r="B563" t="inlineStr">
+        <is>
+          <t>origine_donnee</t>
+        </is>
+      </c>
+      <c r="C563" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D563" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="564">
+      <c r="A564" t="inlineStr">
+        <is>
+          <t>point_service</t>
+        </is>
+      </c>
+      <c r="B564" t="inlineStr">
+        <is>
+          <t>point_service</t>
+        </is>
+      </c>
+      <c r="C564" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D564" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="565">
+      <c r="A565" t="inlineStr">
+        <is>
+          <t>motif</t>
+        </is>
+      </c>
+      <c r="B565" t="inlineStr">
+        <is>
+          <t>motif</t>
+        </is>
+      </c>
+      <c r="C565" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D565" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="566">
+      <c r="A566" t="inlineStr">
+        <is>
+          <t>indicateurs</t>
+        </is>
+      </c>
+      <c r="B566" t="inlineStr">
+        <is>
+          <t>indicateurs</t>
+        </is>
+      </c>
+      <c r="C566" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D566" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="567">
+      <c r="A567" t="inlineStr">
+        <is>
+          <t>reference_liste</t>
+        </is>
+      </c>
+      <c r="B567" t="inlineStr">
+        <is>
+          <t>reference_liste</t>
+        </is>
+      </c>
+      <c r="C567" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D567" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="568">
+      <c r="A568" t="inlineStr">
+        <is>
+          <t>reference_cloture</t>
+        </is>
+      </c>
+      <c r="B568" t="inlineStr">
+        <is>
+          <t>reference_cloture</t>
+        </is>
+      </c>
+      <c r="C568" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D568" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="569">
+      <c r="A569" t="inlineStr">
+        <is>
+          <t>reference_arrete</t>
+        </is>
+      </c>
+      <c r="B569" t="inlineStr">
+        <is>
+          <t>reference_arrete</t>
+        </is>
+      </c>
+      <c r="C569" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D569" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="570">
+      <c r="A570" t="inlineStr">
+        <is>
+          <t>reference_cycle</t>
+        </is>
+      </c>
+      <c r="B570" t="inlineStr">
+        <is>
+          <t>reference_cycle</t>
+        </is>
+      </c>
+      <c r="C570" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D570" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="571">
+      <c r="A571" t="inlineStr">
+        <is>
+          <t>reference_depart</t>
+        </is>
+      </c>
+      <c r="B571" t="inlineStr">
+        <is>
+          <t>reference_depart</t>
+        </is>
+      </c>
+      <c r="C571" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D571" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="572">
+      <c r="A572" t="inlineStr">
+        <is>
+          <t>reference_execution</t>
+        </is>
+      </c>
+      <c r="B572" t="inlineStr">
+        <is>
+          <t>reference_execution</t>
+        </is>
+      </c>
+      <c r="C572" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D572" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="573">
+      <c r="A573" t="inlineStr">
+        <is>
+          <t>reference_mouvement</t>
+        </is>
+      </c>
+      <c r="B573" t="inlineStr">
+        <is>
+          <t>reference_mouvement</t>
+        </is>
+      </c>
+      <c r="C573" t="inlineStr">
+        <is>
+          <t>Conformité</t>
+        </is>
+      </c>
+      <c r="D573" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="574">
+      <c r="A574" t="inlineStr">
+        <is>
+          <t>reference_ecriture</t>
+        </is>
+      </c>
+      <c r="B574" t="inlineStr">
+        <is>
+          <t>piece_id</t>
+        </is>
+      </c>
+      <c r="C574" t="inlineStr">
+        <is>
+          <t>Tous cycles</t>
+        </is>
+      </c>
+      <c r="D574" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="575">
+      <c r="A575" t="inlineStr">
+        <is>
+          <t>reference_compte</t>
+        </is>
+      </c>
+      <c r="B575" t="inlineStr">
+        <is>
+          <t>compte_id</t>
+        </is>
+      </c>
+      <c r="C575" t="inlineStr">
+        <is>
+          <t>Tous cycles</t>
+        </is>
+      </c>
+      <c r="D575" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="576">
+      <c r="A576" t="inlineStr">
+        <is>
+          <t>numero_operation_annulee</t>
+        </is>
+      </c>
+      <c r="B576" t="inlineStr">
+        <is>
+          <t>id_operation_annulee</t>
+        </is>
+      </c>
+      <c r="C576" t="inlineStr">
+        <is>
+          <t>Op?rations</t>
+        </is>
+      </c>
+      <c r="D576" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
+      </c>
+    </row>
+    <row r="577">
+      <c r="A577" t="inlineStr">
+        <is>
+          <t>numero_operation_origine</t>
+        </is>
+      </c>
+      <c r="B577" t="inlineStr">
+        <is>
+          <t>id_operation_mere</t>
+        </is>
+      </c>
+      <c r="C577" t="inlineStr">
+        <is>
+          <t>Op?rations</t>
+        </is>
+      </c>
+      <c r="D577" t="inlineStr">
+        <is>
+          <t>FALSE</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>